<commit_message>
Agregando graficos con matplotlib
</commit_message>
<xml_diff>
--- a/operaciones_crypto2.xlsx
+++ b/operaciones_crypto2.xlsx
@@ -12,6 +12,7 @@
     <sheet name="Operaciones abiertas" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Operaciones cerradas" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Resumen por moneda" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Gráfico PNL por moneda" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -126,6 +127,36 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7620000" cy="4762500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1649,4 +1680,18 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Agregando mas columnas en guardar datos para operaciones cerradas
</commit_message>
<xml_diff>
--- a/operaciones_crypto2.xlsx
+++ b/operaciones_crypto2.xlsx
@@ -12,7 +12,6 @@
     <sheet name="Operaciones abiertas" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Operaciones cerradas" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Resumen por moneda" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Gráfico PNL por moneda" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -127,36 +126,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>0</colOff>
-      <row>1</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="7620000" cy="4762500"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="1" name="Image 1" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -448,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -767,14 +736,14 @@
         <v>30.45994517209869</v>
       </c>
       <c r="G9" t="n">
-        <v>0</v>
+        <v>30.45994517209869</v>
       </c>
       <c r="H9" t="n">
-        <v>30.45994517209869</v>
+        <v>0</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>ABIERTA</t>
+          <t>CERRADA</t>
         </is>
       </c>
     </row>
@@ -802,14 +771,14 @@
         <v>21.47458840372226</v>
       </c>
       <c r="G10" t="n">
-        <v>0</v>
+        <v>21.47458840372226</v>
       </c>
       <c r="H10" t="n">
-        <v>21.47458840372226</v>
+        <v>0</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>ABIERTA</t>
+          <t>CERRADA</t>
         </is>
       </c>
     </row>
@@ -845,6 +814,111 @@
       <c r="I11" t="inlineStr">
         <is>
           <t>CERRADA</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>uni</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>21-06-2026</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>50</v>
+      </c>
+      <c r="E12" t="n">
+        <v>3.083</v>
+      </c>
+      <c r="F12" t="n">
+        <v>16.21796951021732</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" t="n">
+        <v>16.21796951021732</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>ABIERTA</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>ronin</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>23-06-2026</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>50</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.0591</v>
+      </c>
+      <c r="F13" t="n">
+        <v>846.0236886632825</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" t="n">
+        <v>846.0236886632825</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>ABIERTA</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>dot</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>23-06-2026</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>50</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0.899</v>
+      </c>
+      <c r="F14" t="n">
+        <v>55.61735261401557</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" t="n">
+        <v>55.61735261401557</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>ABIERTA</t>
         </is>
       </c>
     </row>
@@ -859,7 +933,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1105,6 +1179,72 @@
       </c>
       <c r="I7" t="n">
         <v>1.463680387409198</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="n">
+        <v>9</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>uni</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>15-06-2026</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>21.47458840372226</v>
+      </c>
+      <c r="F8" t="n">
+        <v>3.007</v>
+      </c>
+      <c r="G8" t="n">
+        <v>64.57408732999284</v>
+      </c>
+      <c r="H8" t="n">
+        <v>59.99999999999999</v>
+      </c>
+      <c r="I8" t="n">
+        <v>4.574087329992842</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>uni</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>16-06-2026</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>30.45994517209869</v>
+      </c>
+      <c r="F9" t="n">
+        <v>3.303</v>
+      </c>
+      <c r="G9" t="n">
+        <v>100.609198903442</v>
+      </c>
+      <c r="H9" t="n">
+        <v>100</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0.609198903441964</v>
       </c>
     </row>
   </sheetData>
@@ -1118,7 +1258,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1275,7 +1415,7 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -1284,23 +1424,23 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>23-05-2026</t>
+          <t>21-06-2026</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="E5" t="n">
-        <v>3.283</v>
+        <v>3.083</v>
       </c>
       <c r="F5" t="n">
-        <v>30.45994517209869</v>
+        <v>16.21796951021732</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>30.45994517209869</v>
+        <v>16.21796951021732</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -1310,34 +1450,69 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>uni</t>
+          <t>ronin</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>02-06-2026</t>
+          <t>23-06-2026</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="E6" t="n">
-        <v>2.794</v>
+        <v>0.0591</v>
       </c>
       <c r="F6" t="n">
-        <v>21.47458840372226</v>
+        <v>846.0236886632825</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>21.47458840372226</v>
+        <v>846.0236886632825</v>
       </c>
       <c r="I6" t="inlineStr">
+        <is>
+          <t>ABIERTA</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>13</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>dot</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>23-06-2026</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>50</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.899</v>
+      </c>
+      <c r="F7" t="n">
+        <v>55.61735261401557</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="n">
+        <v>55.61735261401557</v>
+      </c>
+      <c r="I7" t="inlineStr">
         <is>
           <t>ABIERTA</t>
         </is>
@@ -1354,7 +1529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:M9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1380,25 +1555,45 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>Dólares vendidos</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>Precio de compra</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Precio venta</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
         <is>
           <t>Cantidad comprada</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Cantidad vendida total</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Cantidad restante</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Costo proporcional</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>PNL realizado</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
@@ -1422,18 +1617,30 @@
         <v>200</v>
       </c>
       <c r="E2" t="n">
+        <v>110.6542056074766</v>
+      </c>
+      <c r="F2" t="n">
         <v>1605</v>
       </c>
-      <c r="F2" t="n">
+      <c r="G2" t="n">
+        <v>1776</v>
+      </c>
+      <c r="H2" t="n">
         <v>0.1246105919003115</v>
       </c>
-      <c r="G2" t="n">
+      <c r="I2" t="n">
         <v>0.1246105919003115</v>
       </c>
-      <c r="H2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I2" t="inlineStr">
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" t="n">
+        <v>100</v>
+      </c>
+      <c r="L2" t="n">
+        <v>10.65420560747661</v>
+      </c>
+      <c r="M2" t="inlineStr">
         <is>
           <t>CERRADA</t>
         </is>
@@ -1441,7 +1648,7 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -1454,21 +1661,33 @@
         </is>
       </c>
       <c r="D3" t="n">
+        <v>200</v>
+      </c>
+      <c r="E3" t="n">
+        <v>113.1464174454828</v>
+      </c>
+      <c r="F3" t="n">
+        <v>1605</v>
+      </c>
+      <c r="G3" t="n">
+        <v>1816</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.1246105919003115</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.1246105919003115</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="n">
         <v>100</v>
       </c>
-      <c r="E3" t="n">
-        <v>1569</v>
-      </c>
-      <c r="F3" t="n">
-        <v>0.06373486297004462</v>
-      </c>
-      <c r="G3" t="n">
-        <v>0.06373486297004462</v>
-      </c>
-      <c r="H3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I3" t="inlineStr">
+      <c r="L3" t="n">
+        <v>13.14641744548284</v>
+      </c>
+      <c r="M3" t="inlineStr">
         <is>
           <t>CERRADA</t>
         </is>
@@ -1476,7 +1695,7 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -1485,25 +1704,37 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>06-06-2026</t>
+          <t>05-06-2026</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="E4" t="n">
-        <v>1528</v>
+        <v>109.7514340344168</v>
       </c>
       <c r="F4" t="n">
-        <v>0.03272251308900524</v>
+        <v>1569</v>
       </c>
       <c r="G4" t="n">
-        <v>0.03272251308900524</v>
+        <v>1722</v>
       </c>
       <c r="H4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I4" t="inlineStr">
+        <v>0.06373486297004462</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.06373486297004462</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="n">
+        <v>100</v>
+      </c>
+      <c r="L4" t="n">
+        <v>9.751434034416832</v>
+      </c>
+      <c r="M4" t="inlineStr">
         <is>
           <t>CERRADA</t>
         </is>
@@ -1511,11 +1742,11 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ronin</t>
+          <t>eth</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1527,18 +1758,30 @@
         <v>50</v>
       </c>
       <c r="E5" t="n">
-        <v>0.0624</v>
+        <v>55.23560209424085</v>
       </c>
       <c r="F5" t="n">
-        <v>801.2820512820513</v>
+        <v>1528</v>
       </c>
       <c r="G5" t="n">
-        <v>801.2820512820513</v>
+        <v>1688</v>
       </c>
       <c r="H5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I5" t="inlineStr">
+        <v>0.03272251308900524</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.03272251308900524</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="n">
+        <v>50</v>
+      </c>
+      <c r="L5" t="n">
+        <v>5.235602094240846</v>
+      </c>
+      <c r="M5" t="inlineStr">
         <is>
           <t>CERRADA</t>
         </is>
@@ -1546,34 +1789,187 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
+        <v>7</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ronin</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>06-06-2026</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>50</v>
+      </c>
+      <c r="E6" t="n">
+        <v>51.04166666666667</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.0624</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.06370000000000001</v>
+      </c>
+      <c r="H6" t="n">
+        <v>801.2820512820513</v>
+      </c>
+      <c r="I6" t="n">
+        <v>801.2820512820513</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" t="n">
+        <v>50</v>
+      </c>
+      <c r="L6" t="n">
+        <v>1.041666666666671</v>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>CERRADA</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>8</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>uni</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>23-05-2026</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>100</v>
+      </c>
+      <c r="E7" t="n">
+        <v>100.609198903442</v>
+      </c>
+      <c r="F7" t="n">
+        <v>3.283</v>
+      </c>
+      <c r="G7" t="n">
+        <v>3.303</v>
+      </c>
+      <c r="H7" t="n">
+        <v>30.45994517209869</v>
+      </c>
+      <c r="I7" t="n">
+        <v>30.45994517209869</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" t="n">
+        <v>100</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0.609198903441964</v>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>CERRADA</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>9</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>uni</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>02-06-2026</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>60</v>
+      </c>
+      <c r="E8" t="n">
+        <v>64.57408732999284</v>
+      </c>
+      <c r="F8" t="n">
+        <v>2.794</v>
+      </c>
+      <c r="G8" t="n">
+        <v>3.007</v>
+      </c>
+      <c r="H8" t="n">
+        <v>21.47458840372226</v>
+      </c>
+      <c r="I8" t="n">
+        <v>21.47458840372226</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" t="n">
+        <v>59.99999999999999</v>
+      </c>
+      <c r="L8" t="n">
+        <v>4.574087329992842</v>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>CERRADA</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
         <v>10</v>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>uni</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>05-06-2026</t>
         </is>
       </c>
-      <c r="D6" t="n">
+      <c r="D9" t="n">
         <v>39</v>
       </c>
-      <c r="E6" t="n">
+      <c r="E9" t="n">
+        <v>40.4636803874092</v>
+      </c>
+      <c r="F9" t="n">
         <v>2.478</v>
       </c>
-      <c r="F6" t="n">
+      <c r="G9" t="n">
+        <v>2.571</v>
+      </c>
+      <c r="H9" t="n">
         <v>15.73849878934625</v>
       </c>
-      <c r="G6" t="n">
+      <c r="I9" t="n">
         <v>15.73849878934625</v>
       </c>
-      <c r="H6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I6" t="inlineStr">
+      <c r="J9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" t="n">
+        <v>39</v>
+      </c>
+      <c r="L9" t="n">
+        <v>1.463680387409198</v>
+      </c>
+      <c r="M9" t="inlineStr">
         <is>
           <t>CERRADA</t>
         </is>
@@ -1590,7 +1986,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1649,10 +2045,10 @@
         <v>1.041666666666671</v>
       </c>
       <c r="C3" t="n">
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="D3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E3" t="n">
         <v>1</v>
@@ -1665,33 +2061,38 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1.463680387409198</v>
+        <v>6.646966620844005</v>
       </c>
       <c r="C4" t="n">
-        <v>160</v>
+        <v>50</v>
       </c>
       <c r="D4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E4" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>dot</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" t="n">
+        <v>50</v>
+      </c>
+      <c r="D5" t="n">
         <v>1</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
cambiando y actualizando y agregando boxplot y actualizando pnl por moneda y trades cerrados
</commit_message>
<xml_diff>
--- a/operaciones_crypto2.xlsx
+++ b/operaciones_crypto2.xlsx
@@ -12,6 +12,8 @@
     <sheet name="Operaciones abiertas" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Operaciones cerradas" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Resumen por moneda" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Resumen trades cerrados" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Historial" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -417,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I24"/>
+  <dimension ref="A1:I25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1226,14 +1228,14 @@
         <v>767.8244972577696</v>
       </c>
       <c r="G23" t="n">
-        <v>767.8200000000001</v>
+        <v>767.8244972577696</v>
       </c>
       <c r="H23" t="n">
-        <v>0.004497257769571661</v>
+        <v>0</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>ABIERTA</t>
+          <t>CERRADA</t>
         </is>
       </c>
     </row>
@@ -1267,6 +1269,41 @@
         <v>868.0555555555555</v>
       </c>
       <c r="I24" t="inlineStr">
+        <is>
+          <t>ABIERTA</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>axs</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>08-07-2026</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>50</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0.972</v>
+      </c>
+      <c r="F25" t="n">
+        <v>51.440329218107</v>
+      </c>
+      <c r="G25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" t="n">
+        <v>51.440329218107</v>
+      </c>
+      <c r="I25" t="inlineStr">
         <is>
           <t>ABIERTA</t>
         </is>
@@ -2183,7 +2220,7 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -2192,23 +2229,23 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>30-06-2026</t>
+          <t>7-7-2026</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="E16" t="n">
-        <v>0.0547</v>
+        <v>0.0576</v>
       </c>
       <c r="F16" t="n">
-        <v>767.8244972577696</v>
+        <v>868.0555555555555</v>
       </c>
       <c r="G16" t="n">
-        <v>767.8200000000001</v>
+        <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>0.004497257769571661</v>
+        <v>868.0555555555555</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -2218,32 +2255,32 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ronin</t>
+          <t>axs</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>7-7-2026</t>
+          <t>08-07-2026</t>
         </is>
       </c>
       <c r="D17" t="n">
         <v>50</v>
       </c>
       <c r="E17" t="n">
-        <v>0.0576</v>
+        <v>0.972</v>
       </c>
       <c r="F17" t="n">
-        <v>868.0555555555555</v>
+        <v>51.440329218107</v>
       </c>
       <c r="G17" t="n">
         <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>868.0555555555555</v>
+        <v>51.440329218107</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
@@ -2262,7 +2299,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M9"/>
+  <dimension ref="A1:M10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2703,6 +2740,53 @@
         <v>1.463680387409198</v>
       </c>
       <c r="M9" t="inlineStr">
+        <is>
+          <t>CERRADA</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>22</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ronin</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>30-06-2026</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>42</v>
+      </c>
+      <c r="E10" t="n">
+        <v>47.067366</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.0547</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.0613</v>
+      </c>
+      <c r="H10" t="n">
+        <v>767.8244972577696</v>
+      </c>
+      <c r="I10" t="n">
+        <v>767.8244972577696</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" t="n">
+        <v>41.999754</v>
+      </c>
+      <c r="L10" t="n">
+        <v>5.067611999999997</v>
+      </c>
+      <c r="M10" t="inlineStr">
         <is>
           <t>CERRADA</t>
         </is>
@@ -2719,7 +2803,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2775,16 +2859,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1.041666666666671</v>
+        <v>6.109278666666668</v>
       </c>
       <c r="C3" t="n">
-        <v>200.000246</v>
+        <v>200</v>
       </c>
       <c r="D3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
@@ -2842,6 +2926,1884 @@
       </c>
       <c r="E6" t="n">
         <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>axs</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" t="n">
+        <v>50</v>
+      </c>
+      <c r="D7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ID compra</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Nombre</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>PNL realizado</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Resultado</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Diferencia contra promedio</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>eth</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>23.80062305295945</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>MEJOR TRADE</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>17.35763499431848</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>eth</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>9.751434034416832</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>3.308445975775856</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>eth</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>5.235602094240846</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>-1.207385964400129</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>22</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ronin</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>5.067611999999997</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>-1.375376058640978</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>9</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>uni</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>4.574087329992842</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>-1.868900728648133</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>10</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>uni</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>1.463680387409198</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>-4.979307671231777</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ronin</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>1.041666666666671</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>-5.401321391974305</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>uni</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>0.609198903441964</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>PEOR TRADE</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>-5.833789155199011</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M34"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Fecha registro</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Tipo movimiento</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>ID compra</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>ID venta</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Nombre</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Fecha operacion</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Precio</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Dolares</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Costo proporcional</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>PNL realizado</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Detalle</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>09-07-2026 18:52:53</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>IMPORTACION_COMPRA</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>eth</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>23-05-2026</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>0.04948045522018803</v>
+      </c>
+      <c r="H2" t="n">
+        <v>2021</v>
+      </c>
+      <c r="I2" t="n">
+        <v>100</v>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>ABIERTA</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Compra existente antes de crear historial</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>09-07-2026 18:52:53</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>IMPORTACION_COMPRA</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>eth</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>05-06-2026</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>0.1246105919003115</v>
+      </c>
+      <c r="H3" t="n">
+        <v>1605</v>
+      </c>
+      <c r="I3" t="n">
+        <v>200</v>
+      </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>CERRADA</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Compra existente antes de crear historial</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>09-07-2026 18:52:53</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>IMPORTACION_COMPRA</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>3</v>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>eth</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>05-06-2026</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>0.06373486297004462</v>
+      </c>
+      <c r="H4" t="n">
+        <v>1569</v>
+      </c>
+      <c r="I4" t="n">
+        <v>100</v>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>CERRADA</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Compra existente antes de crear historial</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>09-07-2026 18:52:53</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>IMPORTACION_COMPRA</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>eth</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>06-06-2026</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>0.03272251308900524</v>
+      </c>
+      <c r="H5" t="n">
+        <v>1528</v>
+      </c>
+      <c r="I5" t="n">
+        <v>50</v>
+      </c>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>CERRADA</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Compra existente antes de crear historial</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>09-07-2026 18:52:53</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>IMPORTACION_COMPRA</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>5</v>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>ronin</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>22-05-2026</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>534.1880341880342</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.0936</v>
+      </c>
+      <c r="I6" t="n">
+        <v>50</v>
+      </c>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>ABIERTA</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Compra existente antes de crear historial</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>09-07-2026 18:52:53</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>IMPORTACION_COMPRA</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>6</v>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>ronin</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>30-05-2026</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>636.9426751592357</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.0785</v>
+      </c>
+      <c r="I7" t="n">
+        <v>50</v>
+      </c>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>ABIERTA</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Compra existente antes de crear historial</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>09-07-2026 18:52:53</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>IMPORTACION_COMPRA</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>7</v>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>ronin</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>06-06-2026</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>801.2820512820513</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.0624</v>
+      </c>
+      <c r="I8" t="n">
+        <v>50</v>
+      </c>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>CERRADA</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Compra existente antes de crear historial</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>09-07-2026 18:52:53</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>IMPORTACION_COMPRA</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>8</v>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>uni</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>23-05-2026</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>30.45994517209869</v>
+      </c>
+      <c r="H9" t="n">
+        <v>3.283</v>
+      </c>
+      <c r="I9" t="n">
+        <v>100</v>
+      </c>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>CERRADA</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Compra existente antes de crear historial</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>09-07-2026 18:52:53</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>IMPORTACION_COMPRA</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>9</v>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>uni</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>02-06-2026</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>21.47458840372226</v>
+      </c>
+      <c r="H10" t="n">
+        <v>2.794</v>
+      </c>
+      <c r="I10" t="n">
+        <v>60</v>
+      </c>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>CERRADA</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Compra existente antes de crear historial</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>09-07-2026 18:52:53</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>IMPORTACION_COMPRA</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>10</v>
+      </c>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>uni</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>05-06-2026</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>15.73849878934625</v>
+      </c>
+      <c r="H11" t="n">
+        <v>2.478</v>
+      </c>
+      <c r="I11" t="n">
+        <v>39</v>
+      </c>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>CERRADA</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Compra existente antes de crear historial</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>09-07-2026 18:52:53</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>IMPORTACION_COMPRA</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>11</v>
+      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>uni</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>21-06-2026</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>16.21796951021732</v>
+      </c>
+      <c r="H12" t="n">
+        <v>3.083</v>
+      </c>
+      <c r="I12" t="n">
+        <v>50</v>
+      </c>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>ABIERTA</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Compra existente antes de crear historial</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>09-07-2026 18:52:53</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>IMPORTACION_COMPRA</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>12</v>
+      </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>ronin</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>23-06-2026</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>846.0236886632825</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0.0591</v>
+      </c>
+      <c r="I13" t="n">
+        <v>50</v>
+      </c>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>ABIERTA</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Compra existente antes de crear historial</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>09-07-2026 18:52:53</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>IMPORTACION_COMPRA</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>13</v>
+      </c>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>dot</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>23-06-2026</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>55.61735261401557</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0.899</v>
+      </c>
+      <c r="I14" t="n">
+        <v>50</v>
+      </c>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>ABIERTA</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>Compra existente antes de crear historial</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>09-07-2026 18:52:53</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>IMPORTACION_COMPRA</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>14</v>
+      </c>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>eth</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>24-06-2026</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>0.06169031462060456</v>
+      </c>
+      <c r="H15" t="n">
+        <v>1621</v>
+      </c>
+      <c r="I15" t="n">
+        <v>100</v>
+      </c>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>ABIERTA</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>Compra existente antes de crear historial</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>09-07-2026 18:52:53</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>IMPORTACION_COMPRA</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>15</v>
+      </c>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>eth</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>25-06-2026</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>0.03198976327575176</v>
+      </c>
+      <c r="H16" t="n">
+        <v>1563</v>
+      </c>
+      <c r="I16" t="n">
+        <v>50</v>
+      </c>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>ABIERTA</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>Compra existente antes de crear historial</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>09-07-2026 18:52:53</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>IMPORTACION_COMPRA</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>16</v>
+      </c>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>btc</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>28-06-2026</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>0.0007725898555592879</v>
+      </c>
+      <c r="H17" t="n">
+        <v>59540</v>
+      </c>
+      <c r="I17" t="n">
+        <v>46</v>
+      </c>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>ABIERTA</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>Compra existente antes de crear historial</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>09-07-2026 18:52:53</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>IMPORTACION_COMPRA</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>17</v>
+      </c>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>uni</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>28-06-2026</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>17.28907330567082</v>
+      </c>
+      <c r="H18" t="n">
+        <v>2.892</v>
+      </c>
+      <c r="I18" t="n">
+        <v>50</v>
+      </c>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>ABIERTA</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>Compra existente antes de crear historial</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>09-07-2026 18:52:53</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>IMPORTACION_COMPRA</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>18</v>
+      </c>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>uni</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>30-06-2026</t>
+        </is>
+      </c>
+      <c r="G19" t="n">
+        <v>17.94687724335965</v>
+      </c>
+      <c r="H19" t="n">
+        <v>2.786</v>
+      </c>
+      <c r="I19" t="n">
+        <v>50</v>
+      </c>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>ABIERTA</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>Compra existente antes de crear historial</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>09-07-2026 18:52:53</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>IMPORTACION_COMPRA</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>19</v>
+      </c>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>btc</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>30-06-2026</t>
+        </is>
+      </c>
+      <c r="G20" t="n">
+        <v>0.0008475150857685267</v>
+      </c>
+      <c r="H20" t="n">
+        <v>58996</v>
+      </c>
+      <c r="I20" t="n">
+        <v>50</v>
+      </c>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>ABIERTA</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>Compra existente antes de crear historial</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>09-07-2026 18:52:53</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>IMPORTACION_COMPRA</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>20</v>
+      </c>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>eth</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>30-06-2026</t>
+        </is>
+      </c>
+      <c r="G21" t="n">
+        <v>0.03174603174603174</v>
+      </c>
+      <c r="H21" t="n">
+        <v>1575</v>
+      </c>
+      <c r="I21" t="n">
+        <v>50</v>
+      </c>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>ABIERTA</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>Compra existente antes de crear historial</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>09-07-2026 18:52:53</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>IMPORTACION_COMPRA</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>21</v>
+      </c>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>btc</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>30-06-2026</t>
+        </is>
+      </c>
+      <c r="G22" t="n">
+        <v>0.0008534607834769992</v>
+      </c>
+      <c r="H22" t="n">
+        <v>58585</v>
+      </c>
+      <c r="I22" t="n">
+        <v>50</v>
+      </c>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>ABIERTA</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>Compra existente antes de crear historial</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>09-07-2026 18:52:53</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>IMPORTACION_COMPRA</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>22</v>
+      </c>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>ronin</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>30-06-2026</t>
+        </is>
+      </c>
+      <c r="G23" t="n">
+        <v>767.8244972577696</v>
+      </c>
+      <c r="H23" t="n">
+        <v>0.0547</v>
+      </c>
+      <c r="I23" t="n">
+        <v>42</v>
+      </c>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>CERRADA</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>Compra existente antes de crear historial</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>09-07-2026 18:52:53</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>IMPORTACION_COMPRA</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>23</v>
+      </c>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>ronin</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>7-7-2026</t>
+        </is>
+      </c>
+      <c r="G24" t="n">
+        <v>868.0555555555555</v>
+      </c>
+      <c r="H24" t="n">
+        <v>0.0576</v>
+      </c>
+      <c r="I24" t="n">
+        <v>50</v>
+      </c>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>ABIERTA</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>Compra existente antes de crear historial</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>09-07-2026 18:52:53</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>IMPORTACION_COMPRA</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>24</v>
+      </c>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>axs</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>08-07-2026</t>
+        </is>
+      </c>
+      <c r="G25" t="n">
+        <v>51.440329218107</v>
+      </c>
+      <c r="H25" t="n">
+        <v>0.972</v>
+      </c>
+      <c r="I25" t="n">
+        <v>50</v>
+      </c>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>ABIERTA</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>Compra existente antes de crear historial</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>09-07-2026 18:52:53</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>IMPORTACION_VENTA</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>4</v>
+      </c>
+      <c r="D26" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>eth</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>07-06-2026</t>
+        </is>
+      </c>
+      <c r="G26" t="n">
+        <v>0.03272251308900524</v>
+      </c>
+      <c r="H26" t="n">
+        <v>1688</v>
+      </c>
+      <c r="I26" t="n">
+        <v>55.23560209424085</v>
+      </c>
+      <c r="J26" t="n">
+        <v>50</v>
+      </c>
+      <c r="K26" t="n">
+        <v>5.235602094240846</v>
+      </c>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>Venta existente antes de crear historial</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>09-07-2026 18:52:53</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>IMPORTACION_VENTA</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>3</v>
+      </c>
+      <c r="D27" t="n">
+        <v>2</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>eth</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>14-06-2026</t>
+        </is>
+      </c>
+      <c r="G27" t="n">
+        <v>0.06373486297004462</v>
+      </c>
+      <c r="H27" t="n">
+        <v>1722</v>
+      </c>
+      <c r="I27" t="n">
+        <v>109.7514340344168</v>
+      </c>
+      <c r="J27" t="n">
+        <v>100</v>
+      </c>
+      <c r="K27" t="n">
+        <v>9.751434034416832</v>
+      </c>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>Venta existente antes de crear historial</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>09-07-2026 18:52:53</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>IMPORTACION_VENTA</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>2</v>
+      </c>
+      <c r="D28" t="n">
+        <v>3</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>eth</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>15-06-2026</t>
+        </is>
+      </c>
+      <c r="G28" t="n">
+        <v>0.06230529595015575</v>
+      </c>
+      <c r="H28" t="n">
+        <v>1776</v>
+      </c>
+      <c r="I28" t="n">
+        <v>110.6542056074766</v>
+      </c>
+      <c r="J28" t="n">
+        <v>100</v>
+      </c>
+      <c r="K28" t="n">
+        <v>10.65420560747661</v>
+      </c>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>Venta existente antes de crear historial</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>09-07-2026 18:52:53</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>IMPORTACION_VENTA</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>2</v>
+      </c>
+      <c r="D29" t="n">
+        <v>4</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>eth</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>15-06-2026</t>
+        </is>
+      </c>
+      <c r="G29" t="n">
+        <v>0.06230529595015575</v>
+      </c>
+      <c r="H29" t="n">
+        <v>1816</v>
+      </c>
+      <c r="I29" t="n">
+        <v>113.1464174454828</v>
+      </c>
+      <c r="J29" t="n">
+        <v>100</v>
+      </c>
+      <c r="K29" t="n">
+        <v>13.14641744548284</v>
+      </c>
+      <c r="L29" t="inlineStr"/>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>Venta existente antes de crear historial</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>09-07-2026 18:52:53</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>IMPORTACION_VENTA</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>7</v>
+      </c>
+      <c r="D30" t="n">
+        <v>5</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>ronin</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>25-06-2026</t>
+        </is>
+      </c>
+      <c r="G30" t="n">
+        <v>801.2820512820513</v>
+      </c>
+      <c r="H30" t="n">
+        <v>0.06370000000000001</v>
+      </c>
+      <c r="I30" t="n">
+        <v>51.04166666666667</v>
+      </c>
+      <c r="J30" t="n">
+        <v>50</v>
+      </c>
+      <c r="K30" t="n">
+        <v>1.041666666666671</v>
+      </c>
+      <c r="L30" t="inlineStr"/>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>Venta existente antes de crear historial</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>09-07-2026 18:52:53</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>IMPORTACION_VENTA</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>10</v>
+      </c>
+      <c r="D31" t="n">
+        <v>6</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>uni</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>14-06-2026</t>
+        </is>
+      </c>
+      <c r="G31" t="n">
+        <v>15.73849878934625</v>
+      </c>
+      <c r="H31" t="n">
+        <v>2.571</v>
+      </c>
+      <c r="I31" t="n">
+        <v>40.4636803874092</v>
+      </c>
+      <c r="J31" t="n">
+        <v>39</v>
+      </c>
+      <c r="K31" t="n">
+        <v>1.463680387409198</v>
+      </c>
+      <c r="L31" t="inlineStr"/>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>Venta existente antes de crear historial</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>09-07-2026 18:52:53</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>IMPORTACION_VENTA</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>9</v>
+      </c>
+      <c r="D32" t="n">
+        <v>7</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>uni</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>15-06-2026</t>
+        </is>
+      </c>
+      <c r="G32" t="n">
+        <v>21.47458840372226</v>
+      </c>
+      <c r="H32" t="n">
+        <v>3.007</v>
+      </c>
+      <c r="I32" t="n">
+        <v>64.57408732999284</v>
+      </c>
+      <c r="J32" t="n">
+        <v>59.99999999999999</v>
+      </c>
+      <c r="K32" t="n">
+        <v>4.574087329992842</v>
+      </c>
+      <c r="L32" t="inlineStr"/>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>Venta existente antes de crear historial</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>09-07-2026 18:52:53</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>IMPORTACION_VENTA</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>8</v>
+      </c>
+      <c r="D33" t="n">
+        <v>8</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>uni</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>16-06-2026</t>
+        </is>
+      </c>
+      <c r="G33" t="n">
+        <v>30.45994517209869</v>
+      </c>
+      <c r="H33" t="n">
+        <v>3.303</v>
+      </c>
+      <c r="I33" t="n">
+        <v>100.609198903442</v>
+      </c>
+      <c r="J33" t="n">
+        <v>100</v>
+      </c>
+      <c r="K33" t="n">
+        <v>0.609198903441964</v>
+      </c>
+      <c r="L33" t="inlineStr"/>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>Venta existente antes de crear historial</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>09-07-2026 18:52:53</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>IMPORTACION_VENTA</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>22</v>
+      </c>
+      <c r="D34" t="n">
+        <v>9</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>ronin</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>04-07-2026</t>
+        </is>
+      </c>
+      <c r="G34" t="n">
+        <v>767.8200000000001</v>
+      </c>
+      <c r="H34" t="n">
+        <v>0.0613</v>
+      </c>
+      <c r="I34" t="n">
+        <v>47.067366</v>
+      </c>
+      <c r="J34" t="n">
+        <v>41.999754</v>
+      </c>
+      <c r="K34" t="n">
+        <v>5.067611999999997</v>
+      </c>
+      <c r="L34" t="inlineStr"/>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>Venta existente antes de crear historial</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
mejorando error de en operaciones abiertas que se vea la cantidad comprada si es con muchos decimales ahora se ve bien
</commit_message>
<xml_diff>
--- a/operaciones_crypto2.xlsx
+++ b/operaciones_crypto2.xlsx
@@ -52,8 +52,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -489,14 +490,20 @@
       <c r="E2" t="n">
         <v>2021</v>
       </c>
-      <c r="F2" t="n">
-        <v>0.04948045522018803</v>
-      </c>
-      <c r="G2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H2" t="n">
-        <v>0.04948045522018803</v>
+      <c r="F2" s="1" t="inlineStr">
+        <is>
+          <t>0.04948046</t>
+        </is>
+      </c>
+      <c r="G2" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H2" s="1" t="inlineStr">
+        <is>
+          <t>0.04948046</t>
+        </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -524,14 +531,20 @@
       <c r="E3" t="n">
         <v>1605</v>
       </c>
-      <c r="F3" t="n">
-        <v>0.1246105919003115</v>
-      </c>
-      <c r="G3" t="n">
-        <v>0.1246105919003115</v>
-      </c>
-      <c r="H3" t="n">
-        <v>0</v>
+      <c r="F3" s="1" t="inlineStr">
+        <is>
+          <t>0.12461059</t>
+        </is>
+      </c>
+      <c r="G3" s="1" t="inlineStr">
+        <is>
+          <t>0.12461059</t>
+        </is>
+      </c>
+      <c r="H3" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
@@ -559,14 +572,20 @@
       <c r="E4" t="n">
         <v>1569</v>
       </c>
-      <c r="F4" t="n">
-        <v>0.06373486297004462</v>
-      </c>
-      <c r="G4" t="n">
-        <v>0.06373486297004462</v>
-      </c>
-      <c r="H4" t="n">
-        <v>0</v>
+      <c r="F4" s="1" t="inlineStr">
+        <is>
+          <t>0.06373486</t>
+        </is>
+      </c>
+      <c r="G4" s="1" t="inlineStr">
+        <is>
+          <t>0.06373486</t>
+        </is>
+      </c>
+      <c r="H4" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -594,14 +613,20 @@
       <c r="E5" t="n">
         <v>1528</v>
       </c>
-      <c r="F5" t="n">
-        <v>0.03272251308900524</v>
-      </c>
-      <c r="G5" t="n">
-        <v>0.03272251308900524</v>
-      </c>
-      <c r="H5" t="n">
-        <v>0</v>
+      <c r="F5" s="1" t="inlineStr">
+        <is>
+          <t>0.03272251</t>
+        </is>
+      </c>
+      <c r="G5" s="1" t="inlineStr">
+        <is>
+          <t>0.03272251</t>
+        </is>
+      </c>
+      <c r="H5" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -629,14 +654,20 @@
       <c r="E6" t="n">
         <v>0.0936</v>
       </c>
-      <c r="F6" t="n">
-        <v>534.1880341880342</v>
-      </c>
-      <c r="G6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H6" t="n">
-        <v>534.1880341880342</v>
+      <c r="F6" s="1" t="inlineStr">
+        <is>
+          <t>534.18803419</t>
+        </is>
+      </c>
+      <c r="G6" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H6" s="1" t="inlineStr">
+        <is>
+          <t>534.18803419</t>
+        </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -664,14 +695,20 @@
       <c r="E7" t="n">
         <v>0.0785</v>
       </c>
-      <c r="F7" t="n">
-        <v>636.9426751592357</v>
-      </c>
-      <c r="G7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H7" t="n">
-        <v>636.9426751592357</v>
+      <c r="F7" s="1" t="inlineStr">
+        <is>
+          <t>636.94267516</t>
+        </is>
+      </c>
+      <c r="G7" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H7" s="1" t="inlineStr">
+        <is>
+          <t>636.94267516</t>
+        </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
@@ -699,14 +736,20 @@
       <c r="E8" t="n">
         <v>0.0624</v>
       </c>
-      <c r="F8" t="n">
-        <v>801.2820512820513</v>
-      </c>
-      <c r="G8" t="n">
-        <v>801.2820512820513</v>
-      </c>
-      <c r="H8" t="n">
-        <v>0</v>
+      <c r="F8" s="1" t="inlineStr">
+        <is>
+          <t>801.28205128</t>
+        </is>
+      </c>
+      <c r="G8" s="1" t="inlineStr">
+        <is>
+          <t>801.28205128</t>
+        </is>
+      </c>
+      <c r="H8" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
@@ -734,14 +777,20 @@
       <c r="E9" t="n">
         <v>3.283</v>
       </c>
-      <c r="F9" t="n">
-        <v>30.45994517209869</v>
-      </c>
-      <c r="G9" t="n">
-        <v>30.45994517209869</v>
-      </c>
-      <c r="H9" t="n">
-        <v>0</v>
+      <c r="F9" s="1" t="inlineStr">
+        <is>
+          <t>30.45994517</t>
+        </is>
+      </c>
+      <c r="G9" s="1" t="inlineStr">
+        <is>
+          <t>30.45994517</t>
+        </is>
+      </c>
+      <c r="H9" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
@@ -769,14 +818,20 @@
       <c r="E10" t="n">
         <v>2.794</v>
       </c>
-      <c r="F10" t="n">
-        <v>21.47458840372226</v>
-      </c>
-      <c r="G10" t="n">
-        <v>21.47458840372226</v>
-      </c>
-      <c r="H10" t="n">
-        <v>0</v>
+      <c r="F10" s="1" t="inlineStr">
+        <is>
+          <t>21.4745884</t>
+        </is>
+      </c>
+      <c r="G10" s="1" t="inlineStr">
+        <is>
+          <t>21.4745884</t>
+        </is>
+      </c>
+      <c r="H10" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -804,14 +859,20 @@
       <c r="E11" t="n">
         <v>2.478</v>
       </c>
-      <c r="F11" t="n">
-        <v>15.73849878934625</v>
-      </c>
-      <c r="G11" t="n">
-        <v>15.73849878934625</v>
-      </c>
-      <c r="H11" t="n">
-        <v>0</v>
+      <c r="F11" s="1" t="inlineStr">
+        <is>
+          <t>15.73849879</t>
+        </is>
+      </c>
+      <c r="G11" s="1" t="inlineStr">
+        <is>
+          <t>15.73849879</t>
+        </is>
+      </c>
+      <c r="H11" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
@@ -839,14 +900,20 @@
       <c r="E12" t="n">
         <v>3.083</v>
       </c>
-      <c r="F12" t="n">
-        <v>16.21796951021732</v>
-      </c>
-      <c r="G12" t="n">
-        <v>16.21796951021732</v>
-      </c>
-      <c r="H12" t="n">
-        <v>0</v>
+      <c r="F12" s="1" t="inlineStr">
+        <is>
+          <t>16.21796951</t>
+        </is>
+      </c>
+      <c r="G12" s="1" t="inlineStr">
+        <is>
+          <t>16.21796951</t>
+        </is>
+      </c>
+      <c r="H12" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
@@ -874,14 +941,20 @@
       <c r="E13" t="n">
         <v>0.0591</v>
       </c>
-      <c r="F13" t="n">
-        <v>846.0236886632825</v>
-      </c>
-      <c r="G13" t="n">
-        <v>0</v>
-      </c>
-      <c r="H13" t="n">
-        <v>846.0236886632825</v>
+      <c r="F13" s="1" t="inlineStr">
+        <is>
+          <t>846.02368866</t>
+        </is>
+      </c>
+      <c r="G13" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H13" s="1" t="inlineStr">
+        <is>
+          <t>846.02368866</t>
+        </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
@@ -909,14 +982,20 @@
       <c r="E14" t="n">
         <v>0.899</v>
       </c>
-      <c r="F14" t="n">
-        <v>55.61735261401557</v>
-      </c>
-      <c r="G14" t="n">
-        <v>0</v>
-      </c>
-      <c r="H14" t="n">
-        <v>55.61735261401557</v>
+      <c r="F14" s="1" t="inlineStr">
+        <is>
+          <t>55.61735261</t>
+        </is>
+      </c>
+      <c r="G14" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H14" s="1" t="inlineStr">
+        <is>
+          <t>55.61735261</t>
+        </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
@@ -944,14 +1023,20 @@
       <c r="E15" t="n">
         <v>1621</v>
       </c>
-      <c r="F15" t="n">
-        <v>0.06169031462060456</v>
-      </c>
-      <c r="G15" t="n">
-        <v>0.06169031462060456</v>
-      </c>
-      <c r="H15" t="n">
-        <v>0</v>
+      <c r="F15" s="1" t="inlineStr">
+        <is>
+          <t>0.06169031</t>
+        </is>
+      </c>
+      <c r="G15" s="1" t="inlineStr">
+        <is>
+          <t>0.06169031</t>
+        </is>
+      </c>
+      <c r="H15" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -979,14 +1064,20 @@
       <c r="E16" t="n">
         <v>1563</v>
       </c>
-      <c r="F16" t="n">
-        <v>0.03198976327575176</v>
-      </c>
-      <c r="G16" t="n">
-        <v>0.03198976327575176</v>
-      </c>
-      <c r="H16" t="n">
-        <v>0</v>
+      <c r="F16" s="1" t="inlineStr">
+        <is>
+          <t>0.03198976</t>
+        </is>
+      </c>
+      <c r="G16" s="1" t="inlineStr">
+        <is>
+          <t>0.03198976</t>
+        </is>
+      </c>
+      <c r="H16" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -1014,14 +1105,20 @@
       <c r="E17" t="n">
         <v>59540</v>
       </c>
-      <c r="F17" t="n">
-        <v>0.0007725898555592879</v>
-      </c>
-      <c r="G17" t="n">
-        <v>0</v>
-      </c>
-      <c r="H17" t="n">
-        <v>0.0007725898555592879</v>
+      <c r="F17" s="1" t="inlineStr">
+        <is>
+          <t>0.00077259</t>
+        </is>
+      </c>
+      <c r="G17" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H17" s="1" t="inlineStr">
+        <is>
+          <t>0.00077259</t>
+        </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
@@ -1049,14 +1146,20 @@
       <c r="E18" t="n">
         <v>2.892</v>
       </c>
-      <c r="F18" t="n">
-        <v>17.28907330567082</v>
-      </c>
-      <c r="G18" t="n">
-        <v>17.28907330567082</v>
-      </c>
-      <c r="H18" t="n">
-        <v>0</v>
+      <c r="F18" s="1" t="inlineStr">
+        <is>
+          <t>17.28907331</t>
+        </is>
+      </c>
+      <c r="G18" s="1" t="inlineStr">
+        <is>
+          <t>17.28907331</t>
+        </is>
+      </c>
+      <c r="H18" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
@@ -1084,14 +1187,20 @@
       <c r="E19" t="n">
         <v>2.786</v>
       </c>
-      <c r="F19" t="n">
-        <v>17.94687724335965</v>
-      </c>
-      <c r="G19" t="n">
-        <v>17.94687724335965</v>
-      </c>
-      <c r="H19" t="n">
-        <v>0</v>
+      <c r="F19" s="1" t="inlineStr">
+        <is>
+          <t>17.94687724</t>
+        </is>
+      </c>
+      <c r="G19" s="1" t="inlineStr">
+        <is>
+          <t>17.94687724</t>
+        </is>
+      </c>
+      <c r="H19" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
@@ -1119,14 +1228,20 @@
       <c r="E20" t="n">
         <v>58996</v>
       </c>
-      <c r="F20" t="n">
-        <v>0.0008475150857685267</v>
-      </c>
-      <c r="G20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H20" t="n">
-        <v>0.0008475150857685267</v>
+      <c r="F20" s="1" t="inlineStr">
+        <is>
+          <t>0.00084752</t>
+        </is>
+      </c>
+      <c r="G20" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H20" s="1" t="inlineStr">
+        <is>
+          <t>0.00084752</t>
+        </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
@@ -1154,14 +1269,20 @@
       <c r="E21" t="n">
         <v>1575</v>
       </c>
-      <c r="F21" t="n">
-        <v>0.03174603174603174</v>
-      </c>
-      <c r="G21" t="n">
-        <v>0.03174603174603174</v>
-      </c>
-      <c r="H21" t="n">
-        <v>0</v>
+      <c r="F21" s="1" t="inlineStr">
+        <is>
+          <t>0.03174603</t>
+        </is>
+      </c>
+      <c r="G21" s="1" t="inlineStr">
+        <is>
+          <t>0.03174603</t>
+        </is>
+      </c>
+      <c r="H21" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
@@ -1189,14 +1310,20 @@
       <c r="E22" t="n">
         <v>58585</v>
       </c>
-      <c r="F22" t="n">
-        <v>0.0008534607834769992</v>
-      </c>
-      <c r="G22" t="n">
-        <v>0.0008534607834769992</v>
-      </c>
-      <c r="H22" t="n">
-        <v>0</v>
+      <c r="F22" s="1" t="inlineStr">
+        <is>
+          <t>0.00085346</t>
+        </is>
+      </c>
+      <c r="G22" s="1" t="inlineStr">
+        <is>
+          <t>0.00085346</t>
+        </is>
+      </c>
+      <c r="H22" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
@@ -1224,14 +1351,20 @@
       <c r="E23" t="n">
         <v>0.0547</v>
       </c>
-      <c r="F23" t="n">
-        <v>767.8244972577696</v>
-      </c>
-      <c r="G23" t="n">
-        <v>767.8244972577696</v>
-      </c>
-      <c r="H23" t="n">
-        <v>0</v>
+      <c r="F23" s="1" t="inlineStr">
+        <is>
+          <t>767.82449726</t>
+        </is>
+      </c>
+      <c r="G23" s="1" t="inlineStr">
+        <is>
+          <t>767.82449726</t>
+        </is>
+      </c>
+      <c r="H23" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -1259,14 +1392,20 @@
       <c r="E24" t="n">
         <v>0.0576</v>
       </c>
-      <c r="F24" t="n">
-        <v>868.0555555555555</v>
-      </c>
-      <c r="G24" t="n">
-        <v>0</v>
-      </c>
-      <c r="H24" t="n">
-        <v>868.0555555555555</v>
+      <c r="F24" s="1" t="inlineStr">
+        <is>
+          <t>868.05555556</t>
+        </is>
+      </c>
+      <c r="G24" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H24" s="1" t="inlineStr">
+        <is>
+          <t>868.05555556</t>
+        </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -1294,14 +1433,20 @@
       <c r="E25" t="n">
         <v>0.972</v>
       </c>
-      <c r="F25" t="n">
-        <v>51.440329218107</v>
-      </c>
-      <c r="G25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H25" t="n">
-        <v>51.440329218107</v>
+      <c r="F25" s="1" t="inlineStr">
+        <is>
+          <t>51.44032922</t>
+        </is>
+      </c>
+      <c r="G25" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H25" s="1" t="inlineStr">
+        <is>
+          <t>51.44032922</t>
+        </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
@@ -1387,8 +1532,10 @@
           <t>07-06-2026</t>
         </is>
       </c>
-      <c r="E2" t="n">
-        <v>0.03272251308900524</v>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>0.03272251</t>
+        </is>
       </c>
       <c r="F2" t="n">
         <v>1688</v>
@@ -1420,8 +1567,10 @@
           <t>14-06-2026</t>
         </is>
       </c>
-      <c r="E3" t="n">
-        <v>0.06373486297004462</v>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>0.06373486</t>
+        </is>
       </c>
       <c r="F3" t="n">
         <v>1722</v>
@@ -1453,8 +1602,10 @@
           <t>15-06-2026</t>
         </is>
       </c>
-      <c r="E4" t="n">
-        <v>0.06230529595015575</v>
+      <c r="E4" s="1" t="inlineStr">
+        <is>
+          <t>0.0623053</t>
+        </is>
       </c>
       <c r="F4" t="n">
         <v>1776</v>
@@ -1486,8 +1637,10 @@
           <t>15-06-2026</t>
         </is>
       </c>
-      <c r="E5" t="n">
-        <v>0.06230529595015575</v>
+      <c r="E5" s="1" t="inlineStr">
+        <is>
+          <t>0.0623053</t>
+        </is>
       </c>
       <c r="F5" t="n">
         <v>1816</v>
@@ -1519,8 +1672,10 @@
           <t>25-06-2026</t>
         </is>
       </c>
-      <c r="E6" t="n">
-        <v>801.2820512820513</v>
+      <c r="E6" s="1" t="inlineStr">
+        <is>
+          <t>801.28205128</t>
+        </is>
       </c>
       <c r="F6" t="n">
         <v>0.06370000000000001</v>
@@ -1552,8 +1707,10 @@
           <t>14-06-2026</t>
         </is>
       </c>
-      <c r="E7" t="n">
-        <v>15.73849878934625</v>
+      <c r="E7" s="1" t="inlineStr">
+        <is>
+          <t>15.73849879</t>
+        </is>
       </c>
       <c r="F7" t="n">
         <v>2.571</v>
@@ -1585,8 +1742,10 @@
           <t>15-06-2026</t>
         </is>
       </c>
-      <c r="E8" t="n">
-        <v>21.47458840372226</v>
+      <c r="E8" s="1" t="inlineStr">
+        <is>
+          <t>21.4745884</t>
+        </is>
       </c>
       <c r="F8" t="n">
         <v>3.007</v>
@@ -1618,8 +1777,10 @@
           <t>16-06-2026</t>
         </is>
       </c>
-      <c r="E9" t="n">
-        <v>30.45994517209869</v>
+      <c r="E9" s="1" t="inlineStr">
+        <is>
+          <t>30.45994517</t>
+        </is>
       </c>
       <c r="F9" t="n">
         <v>3.303</v>
@@ -1651,8 +1812,10 @@
           <t>04-07-2026</t>
         </is>
       </c>
-      <c r="E10" t="n">
-        <v>767.8200000000001</v>
+      <c r="E10" s="1" t="inlineStr">
+        <is>
+          <t>767.82</t>
+        </is>
       </c>
       <c r="F10" t="n">
         <v>0.0613</v>
@@ -1684,8 +1847,10 @@
           <t>10-07-2026</t>
         </is>
       </c>
-      <c r="E11" t="n">
-        <v>17.94687724335965</v>
+      <c r="E11" s="1" t="inlineStr">
+        <is>
+          <t>17.94687724</t>
+        </is>
       </c>
       <c r="F11" t="n">
         <v>3.4631</v>
@@ -1717,8 +1882,10 @@
           <t>10-07-2026</t>
         </is>
       </c>
-      <c r="E12" t="n">
-        <v>17.28907330567082</v>
+      <c r="E12" s="1" t="inlineStr">
+        <is>
+          <t>17.28907331</t>
+        </is>
       </c>
       <c r="F12" t="n">
         <v>3.519</v>
@@ -1750,8 +1917,10 @@
           <t>10-07-2026</t>
         </is>
       </c>
-      <c r="E13" t="n">
-        <v>0.03198976327575176</v>
+      <c r="E13" s="1" t="inlineStr">
+        <is>
+          <t>0.03198976</t>
+        </is>
       </c>
       <c r="F13" t="n">
         <v>1777.46</v>
@@ -1783,8 +1952,10 @@
           <t>10-07-2026</t>
         </is>
       </c>
-      <c r="E14" t="n">
-        <v>16.21796951021732</v>
+      <c r="E14" s="1" t="inlineStr">
+        <is>
+          <t>16.21796951</t>
+        </is>
       </c>
       <c r="F14" t="n">
         <v>3.677</v>
@@ -1816,8 +1987,10 @@
           <t>10-07-2026</t>
         </is>
       </c>
-      <c r="E15" t="n">
-        <v>0.03174603174603174</v>
+      <c r="E15" s="1" t="inlineStr">
+        <is>
+          <t>0.03174603</t>
+        </is>
       </c>
       <c r="F15" t="n">
         <v>1777.46</v>
@@ -1849,8 +2022,10 @@
           <t>11-07-2026</t>
         </is>
       </c>
-      <c r="E16" t="n">
-        <v>0.06169031462060456</v>
+      <c r="E16" s="1" t="inlineStr">
+        <is>
+          <t>0.06169031</t>
+        </is>
       </c>
       <c r="F16" t="n">
         <v>1825.64</v>
@@ -1882,8 +2057,10 @@
           <t>11-07-2026</t>
         </is>
       </c>
-      <c r="E17" t="n">
-        <v>0.0008534607834769992</v>
+      <c r="E17" s="1" t="inlineStr">
+        <is>
+          <t>0.00085346</t>
+        </is>
       </c>
       <c r="F17" t="n">
         <v>64312.95</v>
@@ -1979,14 +2156,20 @@
       <c r="E2" t="n">
         <v>2021</v>
       </c>
-      <c r="F2" t="n">
-        <v>0.04948045522018803</v>
-      </c>
-      <c r="G2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H2" t="n">
-        <v>0.04948045522018803</v>
+      <c r="F2" s="1" t="inlineStr">
+        <is>
+          <t>0.04948046</t>
+        </is>
+      </c>
+      <c r="G2" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H2" s="1" t="inlineStr">
+        <is>
+          <t>0.04948046</t>
+        </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -2014,14 +2197,20 @@
       <c r="E3" t="n">
         <v>0.0936</v>
       </c>
-      <c r="F3" t="n">
-        <v>534.1880341880342</v>
-      </c>
-      <c r="G3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H3" t="n">
-        <v>534.1880341880342</v>
+      <c r="F3" s="1" t="inlineStr">
+        <is>
+          <t>534.18803419</t>
+        </is>
+      </c>
+      <c r="G3" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H3" s="1" t="inlineStr">
+        <is>
+          <t>534.18803419</t>
+        </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
@@ -2049,14 +2238,20 @@
       <c r="E4" t="n">
         <v>0.0785</v>
       </c>
-      <c r="F4" t="n">
-        <v>636.9426751592357</v>
-      </c>
-      <c r="G4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H4" t="n">
-        <v>636.9426751592357</v>
+      <c r="F4" s="1" t="inlineStr">
+        <is>
+          <t>636.94267516</t>
+        </is>
+      </c>
+      <c r="G4" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H4" s="1" t="inlineStr">
+        <is>
+          <t>636.94267516</t>
+        </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -2084,14 +2279,20 @@
       <c r="E5" t="n">
         <v>0.0591</v>
       </c>
-      <c r="F5" t="n">
-        <v>846.0236886632825</v>
-      </c>
-      <c r="G5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H5" t="n">
-        <v>846.0236886632825</v>
+      <c r="F5" s="1" t="inlineStr">
+        <is>
+          <t>846.02368866</t>
+        </is>
+      </c>
+      <c r="G5" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H5" s="1" t="inlineStr">
+        <is>
+          <t>846.02368866</t>
+        </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -2119,14 +2320,20 @@
       <c r="E6" t="n">
         <v>0.899</v>
       </c>
-      <c r="F6" t="n">
-        <v>55.61735261401557</v>
-      </c>
-      <c r="G6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H6" t="n">
-        <v>55.61735261401557</v>
+      <c r="F6" s="1" t="inlineStr">
+        <is>
+          <t>55.61735261</t>
+        </is>
+      </c>
+      <c r="G6" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H6" s="1" t="inlineStr">
+        <is>
+          <t>55.61735261</t>
+        </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -2154,14 +2361,20 @@
       <c r="E7" t="n">
         <v>59540</v>
       </c>
-      <c r="F7" t="n">
-        <v>0.0007725898555592879</v>
-      </c>
-      <c r="G7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H7" t="n">
-        <v>0.0007725898555592879</v>
+      <c r="F7" s="1" t="inlineStr">
+        <is>
+          <t>0.00077259</t>
+        </is>
+      </c>
+      <c r="G7" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H7" s="1" t="inlineStr">
+        <is>
+          <t>0.00077259</t>
+        </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
@@ -2189,14 +2402,20 @@
       <c r="E8" t="n">
         <v>58996</v>
       </c>
-      <c r="F8" t="n">
-        <v>0.0008475150857685267</v>
-      </c>
-      <c r="G8" t="n">
-        <v>0</v>
-      </c>
-      <c r="H8" t="n">
-        <v>0.0008475150857685267</v>
+      <c r="F8" s="1" t="inlineStr">
+        <is>
+          <t>0.00084752</t>
+        </is>
+      </c>
+      <c r="G8" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H8" s="1" t="inlineStr">
+        <is>
+          <t>0.00084752</t>
+        </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
@@ -2224,14 +2443,20 @@
       <c r="E9" t="n">
         <v>0.0576</v>
       </c>
-      <c r="F9" t="n">
-        <v>868.0555555555555</v>
-      </c>
-      <c r="G9" t="n">
-        <v>0</v>
-      </c>
-      <c r="H9" t="n">
-        <v>868.0555555555555</v>
+      <c r="F9" s="1" t="inlineStr">
+        <is>
+          <t>868.05555556</t>
+        </is>
+      </c>
+      <c r="G9" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H9" s="1" t="inlineStr">
+        <is>
+          <t>868.05555556</t>
+        </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
@@ -2259,14 +2484,20 @@
       <c r="E10" t="n">
         <v>0.972</v>
       </c>
-      <c r="F10" t="n">
-        <v>51.440329218107</v>
-      </c>
-      <c r="G10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H10" t="n">
-        <v>51.440329218107</v>
+      <c r="F10" s="1" t="inlineStr">
+        <is>
+          <t>51.44032922</t>
+        </is>
+      </c>
+      <c r="G10" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H10" s="1" t="inlineStr">
+        <is>
+          <t>51.44032922</t>
+        </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -2391,14 +2622,20 @@
       <c r="H2" t="n">
         <v>1776</v>
       </c>
-      <c r="I2" t="n">
-        <v>0.1246105919003115</v>
-      </c>
-      <c r="J2" t="n">
-        <v>0.1246105919003115</v>
-      </c>
-      <c r="K2" t="n">
-        <v>0</v>
+      <c r="I2" s="1" t="inlineStr">
+        <is>
+          <t>0.12461059</t>
+        </is>
+      </c>
+      <c r="J2" s="1" t="inlineStr">
+        <is>
+          <t>0.12461059</t>
+        </is>
+      </c>
+      <c r="K2" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="L2" t="n">
         <v>100</v>
@@ -2443,14 +2680,20 @@
       <c r="H3" t="n">
         <v>1816</v>
       </c>
-      <c r="I3" t="n">
-        <v>0.1246105919003115</v>
-      </c>
-      <c r="J3" t="n">
-        <v>0.1246105919003115</v>
-      </c>
-      <c r="K3" t="n">
-        <v>0</v>
+      <c r="I3" s="1" t="inlineStr">
+        <is>
+          <t>0.12461059</t>
+        </is>
+      </c>
+      <c r="J3" s="1" t="inlineStr">
+        <is>
+          <t>0.12461059</t>
+        </is>
+      </c>
+      <c r="K3" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="L3" t="n">
         <v>100</v>
@@ -2495,14 +2738,20 @@
       <c r="H4" t="n">
         <v>1722</v>
       </c>
-      <c r="I4" t="n">
-        <v>0.06373486297004462</v>
-      </c>
-      <c r="J4" t="n">
-        <v>0.06373486297004462</v>
-      </c>
-      <c r="K4" t="n">
-        <v>0</v>
+      <c r="I4" s="1" t="inlineStr">
+        <is>
+          <t>0.06373486</t>
+        </is>
+      </c>
+      <c r="J4" s="1" t="inlineStr">
+        <is>
+          <t>0.06373486</t>
+        </is>
+      </c>
+      <c r="K4" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="L4" t="n">
         <v>100</v>
@@ -2547,14 +2796,20 @@
       <c r="H5" t="n">
         <v>1688</v>
       </c>
-      <c r="I5" t="n">
-        <v>0.03272251308900524</v>
-      </c>
-      <c r="J5" t="n">
-        <v>0.03272251308900524</v>
-      </c>
-      <c r="K5" t="n">
-        <v>0</v>
+      <c r="I5" s="1" t="inlineStr">
+        <is>
+          <t>0.03272251</t>
+        </is>
+      </c>
+      <c r="J5" s="1" t="inlineStr">
+        <is>
+          <t>0.03272251</t>
+        </is>
+      </c>
+      <c r="K5" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="L5" t="n">
         <v>50</v>
@@ -2599,14 +2854,20 @@
       <c r="H6" t="n">
         <v>0.06370000000000001</v>
       </c>
-      <c r="I6" t="n">
-        <v>801.2820512820513</v>
-      </c>
-      <c r="J6" t="n">
-        <v>801.2820512820513</v>
-      </c>
-      <c r="K6" t="n">
-        <v>0</v>
+      <c r="I6" s="1" t="inlineStr">
+        <is>
+          <t>801.28205128</t>
+        </is>
+      </c>
+      <c r="J6" s="1" t="inlineStr">
+        <is>
+          <t>801.28205128</t>
+        </is>
+      </c>
+      <c r="K6" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="L6" t="n">
         <v>50</v>
@@ -2651,14 +2912,20 @@
       <c r="H7" t="n">
         <v>3.303</v>
       </c>
-      <c r="I7" t="n">
-        <v>30.45994517209869</v>
-      </c>
-      <c r="J7" t="n">
-        <v>30.45994517209869</v>
-      </c>
-      <c r="K7" t="n">
-        <v>0</v>
+      <c r="I7" s="1" t="inlineStr">
+        <is>
+          <t>30.45994517</t>
+        </is>
+      </c>
+      <c r="J7" s="1" t="inlineStr">
+        <is>
+          <t>30.45994517</t>
+        </is>
+      </c>
+      <c r="K7" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="L7" t="n">
         <v>100</v>
@@ -2703,14 +2970,20 @@
       <c r="H8" t="n">
         <v>3.007</v>
       </c>
-      <c r="I8" t="n">
-        <v>21.47458840372226</v>
-      </c>
-      <c r="J8" t="n">
-        <v>21.47458840372226</v>
-      </c>
-      <c r="K8" t="n">
-        <v>0</v>
+      <c r="I8" s="1" t="inlineStr">
+        <is>
+          <t>21.4745884</t>
+        </is>
+      </c>
+      <c r="J8" s="1" t="inlineStr">
+        <is>
+          <t>21.4745884</t>
+        </is>
+      </c>
+      <c r="K8" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="L8" t="n">
         <v>59.99999999999999</v>
@@ -2755,14 +3028,20 @@
       <c r="H9" t="n">
         <v>2.571</v>
       </c>
-      <c r="I9" t="n">
-        <v>15.73849878934625</v>
-      </c>
-      <c r="J9" t="n">
-        <v>15.73849878934625</v>
-      </c>
-      <c r="K9" t="n">
-        <v>0</v>
+      <c r="I9" s="1" t="inlineStr">
+        <is>
+          <t>15.73849879</t>
+        </is>
+      </c>
+      <c r="J9" s="1" t="inlineStr">
+        <is>
+          <t>15.73849879</t>
+        </is>
+      </c>
+      <c r="K9" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="L9" t="n">
         <v>39</v>
@@ -2807,14 +3086,20 @@
       <c r="H10" t="n">
         <v>3.677</v>
       </c>
-      <c r="I10" t="n">
-        <v>16.21796951021732</v>
-      </c>
-      <c r="J10" t="n">
-        <v>16.21796951021732</v>
-      </c>
-      <c r="K10" t="n">
-        <v>0</v>
+      <c r="I10" s="1" t="inlineStr">
+        <is>
+          <t>16.21796951</t>
+        </is>
+      </c>
+      <c r="J10" s="1" t="inlineStr">
+        <is>
+          <t>16.21796951</t>
+        </is>
+      </c>
+      <c r="K10" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="L10" t="n">
         <v>50</v>
@@ -2859,14 +3144,20 @@
       <c r="H11" t="n">
         <v>1825.64</v>
       </c>
-      <c r="I11" t="n">
-        <v>0.06169031462060456</v>
-      </c>
-      <c r="J11" t="n">
-        <v>0.06169031462060456</v>
-      </c>
-      <c r="K11" t="n">
-        <v>0</v>
+      <c r="I11" s="1" t="inlineStr">
+        <is>
+          <t>0.06169031</t>
+        </is>
+      </c>
+      <c r="J11" s="1" t="inlineStr">
+        <is>
+          <t>0.06169031</t>
+        </is>
+      </c>
+      <c r="K11" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="L11" t="n">
         <v>100</v>
@@ -2911,14 +3202,20 @@
       <c r="H12" t="n">
         <v>1777.46</v>
       </c>
-      <c r="I12" t="n">
-        <v>0.03198976327575176</v>
-      </c>
-      <c r="J12" t="n">
-        <v>0.03198976327575176</v>
-      </c>
-      <c r="K12" t="n">
-        <v>0</v>
+      <c r="I12" s="1" t="inlineStr">
+        <is>
+          <t>0.03198976</t>
+        </is>
+      </c>
+      <c r="J12" s="1" t="inlineStr">
+        <is>
+          <t>0.03198976</t>
+        </is>
+      </c>
+      <c r="K12" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="L12" t="n">
         <v>50</v>
@@ -2963,14 +3260,20 @@
       <c r="H13" t="n">
         <v>3.519</v>
       </c>
-      <c r="I13" t="n">
-        <v>17.28907330567082</v>
-      </c>
-      <c r="J13" t="n">
-        <v>17.28907330567082</v>
-      </c>
-      <c r="K13" t="n">
-        <v>0</v>
+      <c r="I13" s="1" t="inlineStr">
+        <is>
+          <t>17.28907331</t>
+        </is>
+      </c>
+      <c r="J13" s="1" t="inlineStr">
+        <is>
+          <t>17.28907331</t>
+        </is>
+      </c>
+      <c r="K13" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="L13" t="n">
         <v>50</v>
@@ -3015,14 +3318,20 @@
       <c r="H14" t="n">
         <v>3.4631</v>
       </c>
-      <c r="I14" t="n">
-        <v>17.94687724335965</v>
-      </c>
-      <c r="J14" t="n">
-        <v>17.94687724335965</v>
-      </c>
-      <c r="K14" t="n">
-        <v>0</v>
+      <c r="I14" s="1" t="inlineStr">
+        <is>
+          <t>17.94687724</t>
+        </is>
+      </c>
+      <c r="J14" s="1" t="inlineStr">
+        <is>
+          <t>17.94687724</t>
+        </is>
+      </c>
+      <c r="K14" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="L14" t="n">
         <v>50</v>
@@ -3067,14 +3376,20 @@
       <c r="H15" t="n">
         <v>1777.46</v>
       </c>
-      <c r="I15" t="n">
-        <v>0.03174603174603174</v>
-      </c>
-      <c r="J15" t="n">
-        <v>0.03174603174603174</v>
-      </c>
-      <c r="K15" t="n">
-        <v>0</v>
+      <c r="I15" s="1" t="inlineStr">
+        <is>
+          <t>0.03174603</t>
+        </is>
+      </c>
+      <c r="J15" s="1" t="inlineStr">
+        <is>
+          <t>0.03174603</t>
+        </is>
+      </c>
+      <c r="K15" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="L15" t="n">
         <v>50</v>
@@ -3119,14 +3434,20 @@
       <c r="H16" t="n">
         <v>64312.95</v>
       </c>
-      <c r="I16" t="n">
-        <v>0.0008534607834769992</v>
-      </c>
-      <c r="J16" t="n">
-        <v>0.0008534607834769992</v>
-      </c>
-      <c r="K16" t="n">
-        <v>0</v>
+      <c r="I16" s="1" t="inlineStr">
+        <is>
+          <t>0.00085346</t>
+        </is>
+      </c>
+      <c r="J16" s="1" t="inlineStr">
+        <is>
+          <t>0.00085346</t>
+        </is>
+      </c>
+      <c r="K16" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="L16" t="n">
         <v>50</v>
@@ -3171,14 +3492,20 @@
       <c r="H17" t="n">
         <v>0.0613</v>
       </c>
-      <c r="I17" t="n">
-        <v>767.8244972577696</v>
-      </c>
-      <c r="J17" t="n">
-        <v>767.8244972577696</v>
-      </c>
-      <c r="K17" t="n">
-        <v>0</v>
+      <c r="I17" s="1" t="inlineStr">
+        <is>
+          <t>767.82449726</t>
+        </is>
+      </c>
+      <c r="J17" s="1" t="inlineStr">
+        <is>
+          <t>767.82449726</t>
+        </is>
+      </c>
+      <c r="K17" s="1" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="L17" t="n">
         <v>41.999754</v>
@@ -3809,8 +4136,10 @@
           <t>23-05-2026</t>
         </is>
       </c>
-      <c r="G2" t="n">
-        <v>0.04948045522018803</v>
+      <c r="G2" s="1" t="inlineStr">
+        <is>
+          <t>0.04948046</t>
+        </is>
       </c>
       <c r="H2" t="n">
         <v>2021</v>
@@ -3856,8 +4185,10 @@
           <t>05-06-2026</t>
         </is>
       </c>
-      <c r="G3" t="n">
-        <v>0.1246105919003115</v>
+      <c r="G3" s="1" t="inlineStr">
+        <is>
+          <t>0.12461059</t>
+        </is>
       </c>
       <c r="H3" t="n">
         <v>1605</v>
@@ -3903,8 +4234,10 @@
           <t>05-06-2026</t>
         </is>
       </c>
-      <c r="G4" t="n">
-        <v>0.06373486297004462</v>
+      <c r="G4" s="1" t="inlineStr">
+        <is>
+          <t>0.06373486</t>
+        </is>
       </c>
       <c r="H4" t="n">
         <v>1569</v>
@@ -3950,8 +4283,10 @@
           <t>06-06-2026</t>
         </is>
       </c>
-      <c r="G5" t="n">
-        <v>0.03272251308900524</v>
+      <c r="G5" s="1" t="inlineStr">
+        <is>
+          <t>0.03272251</t>
+        </is>
       </c>
       <c r="H5" t="n">
         <v>1528</v>
@@ -3997,8 +4332,10 @@
           <t>22-05-2026</t>
         </is>
       </c>
-      <c r="G6" t="n">
-        <v>534.1880341880342</v>
+      <c r="G6" s="1" t="inlineStr">
+        <is>
+          <t>534.18803419</t>
+        </is>
       </c>
       <c r="H6" t="n">
         <v>0.0936</v>
@@ -4044,8 +4381,10 @@
           <t>30-05-2026</t>
         </is>
       </c>
-      <c r="G7" t="n">
-        <v>636.9426751592357</v>
+      <c r="G7" s="1" t="inlineStr">
+        <is>
+          <t>636.94267516</t>
+        </is>
       </c>
       <c r="H7" t="n">
         <v>0.0785</v>
@@ -4091,8 +4430,10 @@
           <t>06-06-2026</t>
         </is>
       </c>
-      <c r="G8" t="n">
-        <v>801.2820512820513</v>
+      <c r="G8" s="1" t="inlineStr">
+        <is>
+          <t>801.28205128</t>
+        </is>
       </c>
       <c r="H8" t="n">
         <v>0.0624</v>
@@ -4138,8 +4479,10 @@
           <t>23-05-2026</t>
         </is>
       </c>
-      <c r="G9" t="n">
-        <v>30.45994517209869</v>
+      <c r="G9" s="1" t="inlineStr">
+        <is>
+          <t>30.45994517</t>
+        </is>
       </c>
       <c r="H9" t="n">
         <v>3.283</v>
@@ -4185,8 +4528,10 @@
           <t>02-06-2026</t>
         </is>
       </c>
-      <c r="G10" t="n">
-        <v>21.47458840372226</v>
+      <c r="G10" s="1" t="inlineStr">
+        <is>
+          <t>21.4745884</t>
+        </is>
       </c>
       <c r="H10" t="n">
         <v>2.794</v>
@@ -4232,8 +4577,10 @@
           <t>05-06-2026</t>
         </is>
       </c>
-      <c r="G11" t="n">
-        <v>15.73849878934625</v>
+      <c r="G11" s="1" t="inlineStr">
+        <is>
+          <t>15.73849879</t>
+        </is>
       </c>
       <c r="H11" t="n">
         <v>2.478</v>
@@ -4279,8 +4626,10 @@
           <t>21-06-2026</t>
         </is>
       </c>
-      <c r="G12" t="n">
-        <v>16.21796951021732</v>
+      <c r="G12" s="1" t="inlineStr">
+        <is>
+          <t>16.21796951</t>
+        </is>
       </c>
       <c r="H12" t="n">
         <v>3.083</v>
@@ -4326,8 +4675,10 @@
           <t>23-06-2026</t>
         </is>
       </c>
-      <c r="G13" t="n">
-        <v>846.0236886632825</v>
+      <c r="G13" s="1" t="inlineStr">
+        <is>
+          <t>846.02368866</t>
+        </is>
       </c>
       <c r="H13" t="n">
         <v>0.0591</v>
@@ -4373,8 +4724,10 @@
           <t>23-06-2026</t>
         </is>
       </c>
-      <c r="G14" t="n">
-        <v>55.61735261401557</v>
+      <c r="G14" s="1" t="inlineStr">
+        <is>
+          <t>55.61735261</t>
+        </is>
       </c>
       <c r="H14" t="n">
         <v>0.899</v>
@@ -4420,8 +4773,10 @@
           <t>24-06-2026</t>
         </is>
       </c>
-      <c r="G15" t="n">
-        <v>0.06169031462060456</v>
+      <c r="G15" s="1" t="inlineStr">
+        <is>
+          <t>0.06169031</t>
+        </is>
       </c>
       <c r="H15" t="n">
         <v>1621</v>
@@ -4467,8 +4822,10 @@
           <t>25-06-2026</t>
         </is>
       </c>
-      <c r="G16" t="n">
-        <v>0.03198976327575176</v>
+      <c r="G16" s="1" t="inlineStr">
+        <is>
+          <t>0.03198976</t>
+        </is>
       </c>
       <c r="H16" t="n">
         <v>1563</v>
@@ -4514,8 +4871,10 @@
           <t>28-06-2026</t>
         </is>
       </c>
-      <c r="G17" t="n">
-        <v>0.0007725898555592879</v>
+      <c r="G17" s="1" t="inlineStr">
+        <is>
+          <t>0.00077259</t>
+        </is>
       </c>
       <c r="H17" t="n">
         <v>59540</v>
@@ -4561,8 +4920,10 @@
           <t>28-06-2026</t>
         </is>
       </c>
-      <c r="G18" t="n">
-        <v>17.28907330567082</v>
+      <c r="G18" s="1" t="inlineStr">
+        <is>
+          <t>17.28907331</t>
+        </is>
       </c>
       <c r="H18" t="n">
         <v>2.892</v>
@@ -4608,8 +4969,10 @@
           <t>30-06-2026</t>
         </is>
       </c>
-      <c r="G19" t="n">
-        <v>17.94687724335965</v>
+      <c r="G19" s="1" t="inlineStr">
+        <is>
+          <t>17.94687724</t>
+        </is>
       </c>
       <c r="H19" t="n">
         <v>2.786</v>
@@ -4655,8 +5018,10 @@
           <t>30-06-2026</t>
         </is>
       </c>
-      <c r="G20" t="n">
-        <v>0.0008475150857685267</v>
+      <c r="G20" s="1" t="inlineStr">
+        <is>
+          <t>0.00084752</t>
+        </is>
       </c>
       <c r="H20" t="n">
         <v>58996</v>
@@ -4702,8 +5067,10 @@
           <t>30-06-2026</t>
         </is>
       </c>
-      <c r="G21" t="n">
-        <v>0.03174603174603174</v>
+      <c r="G21" s="1" t="inlineStr">
+        <is>
+          <t>0.03174603</t>
+        </is>
       </c>
       <c r="H21" t="n">
         <v>1575</v>
@@ -4749,8 +5116,10 @@
           <t>30-06-2026</t>
         </is>
       </c>
-      <c r="G22" t="n">
-        <v>0.0008534607834769992</v>
+      <c r="G22" s="1" t="inlineStr">
+        <is>
+          <t>0.00085346</t>
+        </is>
       </c>
       <c r="H22" t="n">
         <v>58585</v>
@@ -4796,8 +5165,10 @@
           <t>30-06-2026</t>
         </is>
       </c>
-      <c r="G23" t="n">
-        <v>767.8244972577696</v>
+      <c r="G23" s="1" t="inlineStr">
+        <is>
+          <t>767.82449726</t>
+        </is>
       </c>
       <c r="H23" t="n">
         <v>0.0547</v>
@@ -4843,8 +5214,10 @@
           <t>7-7-2026</t>
         </is>
       </c>
-      <c r="G24" t="n">
-        <v>868.0555555555555</v>
+      <c r="G24" s="1" t="inlineStr">
+        <is>
+          <t>868.05555556</t>
+        </is>
       </c>
       <c r="H24" t="n">
         <v>0.0576</v>
@@ -4890,8 +5263,10 @@
           <t>08-07-2026</t>
         </is>
       </c>
-      <c r="G25" t="n">
-        <v>51.440329218107</v>
+      <c r="G25" s="1" t="inlineStr">
+        <is>
+          <t>51.44032922</t>
+        </is>
       </c>
       <c r="H25" t="n">
         <v>0.972</v>
@@ -4939,8 +5314,10 @@
           <t>07-06-2026</t>
         </is>
       </c>
-      <c r="G26" t="n">
-        <v>0.03272251308900524</v>
+      <c r="G26" s="1" t="inlineStr">
+        <is>
+          <t>0.03272251</t>
+        </is>
       </c>
       <c r="H26" t="n">
         <v>1688</v>
@@ -4988,8 +5365,10 @@
           <t>14-06-2026</t>
         </is>
       </c>
-      <c r="G27" t="n">
-        <v>0.06373486297004462</v>
+      <c r="G27" s="1" t="inlineStr">
+        <is>
+          <t>0.06373486</t>
+        </is>
       </c>
       <c r="H27" t="n">
         <v>1722</v>
@@ -5037,8 +5416,10 @@
           <t>15-06-2026</t>
         </is>
       </c>
-      <c r="G28" t="n">
-        <v>0.06230529595015575</v>
+      <c r="G28" s="1" t="inlineStr">
+        <is>
+          <t>0.0623053</t>
+        </is>
       </c>
       <c r="H28" t="n">
         <v>1776</v>
@@ -5086,8 +5467,10 @@
           <t>15-06-2026</t>
         </is>
       </c>
-      <c r="G29" t="n">
-        <v>0.06230529595015575</v>
+      <c r="G29" s="1" t="inlineStr">
+        <is>
+          <t>0.0623053</t>
+        </is>
       </c>
       <c r="H29" t="n">
         <v>1816</v>
@@ -5135,8 +5518,10 @@
           <t>25-06-2026</t>
         </is>
       </c>
-      <c r="G30" t="n">
-        <v>801.2820512820513</v>
+      <c r="G30" s="1" t="inlineStr">
+        <is>
+          <t>801.28205128</t>
+        </is>
       </c>
       <c r="H30" t="n">
         <v>0.06370000000000001</v>
@@ -5184,8 +5569,10 @@
           <t>14-06-2026</t>
         </is>
       </c>
-      <c r="G31" t="n">
-        <v>15.73849878934625</v>
+      <c r="G31" s="1" t="inlineStr">
+        <is>
+          <t>15.73849879</t>
+        </is>
       </c>
       <c r="H31" t="n">
         <v>2.571</v>
@@ -5233,8 +5620,10 @@
           <t>15-06-2026</t>
         </is>
       </c>
-      <c r="G32" t="n">
-        <v>21.47458840372226</v>
+      <c r="G32" s="1" t="inlineStr">
+        <is>
+          <t>21.4745884</t>
+        </is>
       </c>
       <c r="H32" t="n">
         <v>3.007</v>
@@ -5282,8 +5671,10 @@
           <t>16-06-2026</t>
         </is>
       </c>
-      <c r="G33" t="n">
-        <v>30.45994517209869</v>
+      <c r="G33" s="1" t="inlineStr">
+        <is>
+          <t>30.45994517</t>
+        </is>
       </c>
       <c r="H33" t="n">
         <v>3.303</v>
@@ -5331,8 +5722,10 @@
           <t>04-07-2026</t>
         </is>
       </c>
-      <c r="G34" t="n">
-        <v>767.8200000000001</v>
+      <c r="G34" s="1" t="inlineStr">
+        <is>
+          <t>767.82</t>
+        </is>
       </c>
       <c r="H34" t="n">
         <v>0.0613</v>
@@ -5380,8 +5773,10 @@
           <t>10-07-2026</t>
         </is>
       </c>
-      <c r="G35" t="n">
-        <v>17.94687724335965</v>
+      <c r="G35" s="1" t="inlineStr">
+        <is>
+          <t>17.94687724</t>
+        </is>
       </c>
       <c r="H35" t="n">
         <v>3.4631</v>
@@ -5433,8 +5828,10 @@
           <t>10-07-2026</t>
         </is>
       </c>
-      <c r="G36" t="n">
-        <v>17.28907330567082</v>
+      <c r="G36" s="1" t="inlineStr">
+        <is>
+          <t>17.28907331</t>
+        </is>
       </c>
       <c r="H36" t="n">
         <v>3.519</v>
@@ -5486,8 +5883,10 @@
           <t>10-07-2026</t>
         </is>
       </c>
-      <c r="G37" t="n">
-        <v>0.03198976327575176</v>
+      <c r="G37" s="1" t="inlineStr">
+        <is>
+          <t>0.03198976</t>
+        </is>
       </c>
       <c r="H37" t="n">
         <v>1777.46</v>
@@ -5539,8 +5938,10 @@
           <t>10-07-2026</t>
         </is>
       </c>
-      <c r="G38" t="n">
-        <v>16.21796951021732</v>
+      <c r="G38" s="1" t="inlineStr">
+        <is>
+          <t>16.21796951</t>
+        </is>
       </c>
       <c r="H38" t="n">
         <v>3.677</v>
@@ -5592,8 +5993,10 @@
           <t>10-07-2026</t>
         </is>
       </c>
-      <c r="G39" t="n">
-        <v>0.03174603174603174</v>
+      <c r="G39" s="1" t="inlineStr">
+        <is>
+          <t>0.03174603</t>
+        </is>
       </c>
       <c r="H39" t="n">
         <v>1777.46</v>
@@ -5645,8 +6048,10 @@
           <t>11-07-2026</t>
         </is>
       </c>
-      <c r="G40" t="n">
-        <v>0.06169031462060456</v>
+      <c r="G40" s="1" t="inlineStr">
+        <is>
+          <t>0.06169031</t>
+        </is>
       </c>
       <c r="H40" t="n">
         <v>1825.64</v>
@@ -5698,8 +6103,10 @@
           <t>11-07-2026</t>
         </is>
       </c>
-      <c r="G41" t="n">
-        <v>0.0008534607834769992</v>
+      <c r="G41" s="1" t="inlineStr">
+        <is>
+          <t>0.00085346</t>
+        </is>
       </c>
       <c r="H41" t="n">
         <v>64312.95</v>

</xml_diff>